<commit_message>
Actualizar planilla de inscripcion Excel con dorsales asignados y 57 jugadores de Supabase
</commit_message>
<xml_diff>
--- a/public/documentos/Planilla_Inscripcion_Torneo_Juvenil.xlsx
+++ b/public/documentos/Planilla_Inscripcion_Torneo_Juvenil.xlsx
@@ -508,14 +508,14 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G69"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -559,7 +559,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Total Jugadores Registrados en Base de Datos: 57</t>
+          <t>Total Jugadores Inscritos en Base de Datos: 57</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Posición</t>
+          <t>Categoría / Posición</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -607,23 +607,27 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>JUAN JOSE TOBIAS BORNACHERA</t>
+          <t>MIGUEL ANGEL ALDANA CHARRIS</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>1065136281</t>
+          <t>1143249663</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>2013-09-25</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr"/>
+          <t>2012-01-19</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>2013</t>
+          <t>2012</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -638,20 +642,24 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>JAIR ANDRES MORENO ELLES</t>
+          <t>JHOYFRAN DE LOS REYES HILLEMBRAND</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>1194976006</t>
+          <t>1143256788</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>2016-02-16</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr"/>
+          <t>2014-01-05</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
           <t>2014/15/16</t>
@@ -669,23 +677,27 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>ENDERSON MARCANO</t>
+          <t>DANIEL ISAAC RODRÍGUEZ CANTILLO</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>T001</t>
+          <t>1143251275</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr"/>
+          <t>2012-06-05</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>2014/15/16</t>
+          <t>2012</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -700,20 +712,24 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>SEBASTIAN MATHIAS LUGO JIMENEZ</t>
+          <t>JHONIER ARLES RONDON LUNA</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>1043479873</t>
+          <t>1098763962</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>2012-06-28</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr"/>
+          <t>2012-12-07</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
           <t>2012</t>
@@ -731,23 +747,27 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>CESC CRISTIANO SISON HILLENBRAND</t>
+          <t>JOSE MIGUEL ALVAREZ CARRILLO</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>1146538625</t>
+          <t>1143252740</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>2013-11-22</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr"/>
+          <t>2012-05-20</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>2013</t>
+          <t>2012</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -762,23 +782,27 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>JUAN CARLOS HENRIQUEZ MOLINA</t>
+          <t>SANTIAGO ANDRES MENDOZA COLMENAREZ</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>10216012014</t>
+          <t>9062012266</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>2014-01-06</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr"/>
+          <t>2012-06-09</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>2014/15/16</t>
+          <t>2012</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -793,23 +817,27 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>ISRAEL CAMAÑO</t>
+          <t>JUAN JOSE TOBIAS BORNACHERA</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>1015016001</t>
+          <t>1065136281</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr"/>
+          <t>2013-09-25</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>2014/15/16</t>
+          <t>2013</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -824,23 +852,27 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>JOSEP DAVID ALDANA PUERTAS</t>
+          <t>MAYCOL ANDRES VILLAR CUBILLOS</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>1043462171</t>
+          <t>1046711979</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>2013-03-05</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr"/>
+          <t>2012-04-11</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>2013</t>
+          <t>2012</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -855,23 +887,27 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>MATEO DE JESUS BOSCAN GELVEZ</t>
+          <t>DYLAN ALEJANDRO SÁNCHEZ CESPEDES</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>1124517321</t>
+          <t>30528122012</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>2013-09-10</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr"/>
+          <t>2012-12-28</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>2013</t>
+          <t>2012</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -886,20 +922,24 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>DANY JOSE TAPIA SIERRA</t>
+          <t>NELSON PAULINE</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>1137534185</t>
+          <t>5184698</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>2013-05-05</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="inlineStr"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
           <t>2013</t>
@@ -917,20 +957,24 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>NELSON PAULINE</t>
+          <t>DANIEL LÓPEZ ROJO</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>5184698</t>
+          <t>1046718667</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr"/>
+          <t>2013-10-04</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
           <t>2013</t>
@@ -948,23 +992,27 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>MOISES EDUARDO CABALLERO CAÑAS</t>
+          <t>ANTONY DAVID ARIZA ZAMORA</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>1045251440</t>
+          <t>04939456</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>2014-01-27</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr"/>
+          <t>2012-02-13</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>2014/15/16</t>
+          <t>2012</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -979,23 +1027,27 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>JESÚS DAVID AVILA ARIZA</t>
+          <t>CESC CRISTIANO SISON HILLENBRAND</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>1194973338</t>
+          <t>1146538625</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr"/>
+          <t>2013-11-22</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>2014/15/16</t>
+          <t>2013</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -1010,20 +1062,24 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>CARLOS ANDRES MORENO GARCIA</t>
+          <t>PEDROZA SNEYDER</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>1043696535</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>2014-12-04</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="inlineStr"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
           <t>2014/15/16</t>
@@ -1041,20 +1097,24 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>JHOYFRAN DE LOS REYES HILLEMBRAND</t>
+          <t>ANDRES ALBERTO SIERRA ARRIETA</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>1143256788</t>
+          <t>1045738584</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>2014-01-05</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr"/>
+          <t>2014-04-25</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
           <t>2014/15/16</t>
@@ -1072,23 +1132,27 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>STEVEN DAVID CABARCAS PEREZ</t>
+          <t>ANGEL DAVID HERNANDEZ HILLEMBRAND</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>1042263783</t>
+          <t>1143254770</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>2012-03-05</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr"/>
+          <t>2013-05-03</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>2012</t>
+          <t>2013</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -1103,23 +1167,27 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>YOJAINER JESUS VERA VILLALOBOS</t>
+          <t>RENE JUNIOR CERPA ALVAREZ</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>300312673</t>
+          <t>1044223163</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>2012-03-03</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr"/>
+          <t>2013-08-15</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>2012</t>
+          <t>2013</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -1134,23 +1202,27 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>MIGUEL ANGEL ALDANA CHARRIS</t>
+          <t>MARIO DE JESUS PEREZ NAVAS</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>1143249663</t>
+          <t>1194972758</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>2012-01-19</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr"/>
+          <t>2014-12-04</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>2012</t>
+          <t>2014/15/16</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -1165,23 +1237,27 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>ELIUTH DAVID MEZA MADERA</t>
+          <t>JESUS ADRIAN TORRES RIOS</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>1047055557</t>
+          <t>1041697767</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>2014-02-22</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr"/>
+          <t>2012-01-20</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>2014/15/16</t>
+          <t>2012</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -1196,20 +1272,24 @@
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>ESTIBEN ENRIQUE GÓMEZ LÓPEZ</t>
+          <t>ABRAHAM EDUARDO PEREZ COLMENAREZ</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>1046720625</t>
+          <t>12003022014</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>2014-02-14</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr"/>
+          <t>2014-02-03</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
           <t>2014/15/16</t>
@@ -1227,20 +1307,24 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>REY DAVID ARRIETA CARO</t>
+          <t>SANTIAGO RAFAEL TOBIAS BORNACHERA</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>1043469465</t>
+          <t>1065131586</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>2015-04-01</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr"/>
+          <t>2013-12-03</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
           <t>2014/15/16</t>
@@ -1258,20 +1342,24 @@
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>MARIO DE JESUS PEREZ NAVAS</t>
+          <t>JAMED AMARANTO</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>1194972758</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>2014-12-04</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="inlineStr"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
           <t>2014/15/16</t>
@@ -1289,20 +1377,24 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>JUAN ANDRES MARTÍNEZ ALVAREZ</t>
+          <t>ISAAC GABRIEL VENTURA SÁNCHEZ</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>1140897161</t>
+          <t>16509022015</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>2016-03-18</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr"/>
+          <t>2015-02-09</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
           <t>2014/15/16</t>
@@ -1320,20 +1412,24 @@
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>ENELDO JOSE TORREGROZA RODRÍGUEZ</t>
+          <t>REY DAVID ARRIETA CARO</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>1079939684</t>
+          <t>1043469465</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>2015-03-17</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="inlineStr"/>
+          <t>2015-04-01</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
           <t>2014/15/16</t>
@@ -1351,20 +1447,24 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>ANDRES ALBERTO SIERRA ARRIETA</t>
+          <t>ELIUTH DAVID MEZA MADERA</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>1045738584</t>
+          <t>1047055557</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>2014-04-25</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr"/>
+          <t>2014-02-22</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
           <t>2014/15/16</t>
@@ -1382,23 +1482,27 @@
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>SANTIAGO RAFAEL TOBIAS BORNACHERA</t>
+          <t>BRAYAN FERNANDEZ</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>1065131586</t>
+          <t>13</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>2013-12-03</t>
-        </is>
-      </c>
-      <c r="E33" s="7" t="inlineStr"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>2014/15/16</t>
+          <t>2013</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -1413,20 +1517,24 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>ABRAHAM EDUARDO PEREZ COLMENAREZ</t>
+          <t>ANDRES DAVID SOCARRAS CADENA</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>12003022014</t>
+          <t>1044655749</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>2014-02-03</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr"/>
+          <t>2015-01-12</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
           <t>2014/15/16</t>
@@ -1444,23 +1552,27 @@
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>ANGEL DAVID HERNANDEZ HILLEMBRAND</t>
+          <t>STEVEN DAVID CABARCAS PEREZ</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>1143254770</t>
+          <t>1042263783</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>2013-05-03</t>
-        </is>
-      </c>
-      <c r="E35" s="7" t="inlineStr"/>
+          <t>2012-03-05</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>2013</t>
+          <t>2012</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -1475,23 +1587,27 @@
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>DANIEL ISAAC RODRÍGUEZ CANTILLO</t>
+          <t>DEMIAN PEDROZA</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>1143251275</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>2012-06-05</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>2012</t>
+          <t>2014/15/16</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
@@ -1506,23 +1622,27 @@
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>OSCAR DAVID LÓPEZ GARCIA</t>
+          <t>ESTIBEN ENRIQUE GÓMEZ LÓPEZ</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>1043459628</t>
+          <t>1046720625</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>2012-08-03</t>
-        </is>
-      </c>
-      <c r="E37" s="7" t="inlineStr"/>
+          <t>2014-02-14</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>2012</t>
+          <t>2014/15/16</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -1537,20 +1657,24 @@
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>ISAAC GABRIEL VENTURA SÁNCHEZ</t>
+          <t>JUAN ANDRES MARTÍNEZ ALVAREZ</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>16509022015</t>
+          <t>1140897161</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>2015-02-09</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr"/>
+          <t>2016-03-18</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
           <t>2014/15/16</t>
@@ -1568,23 +1692,27 @@
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>MAYCOL ANDRES VILLAR CUBILLOS</t>
+          <t>ENELDO JOSE TORREGROZA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>1046711979</t>
+          <t>1079939684</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>2012-04-11</t>
-        </is>
-      </c>
-      <c r="E39" s="7" t="inlineStr"/>
+          <t>2015-03-17</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>2012</t>
+          <t>2014/15/16</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -1599,20 +1727,24 @@
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>JAIR ANDRES MIRANDA CARO</t>
+          <t>LUIS EDUARDO CADENA SUAREZ</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>1047234329</t>
+          <t>1082352203</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>2012-12-13</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr"/>
+          <t>2012-04-23</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
           <t>2012</t>
@@ -1630,20 +1762,24 @@
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>SANTIAGO HERNANDEZ GARCIA</t>
+          <t>JUAN CARLOS HENRIQUEZ MOLINA</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>1043467436</t>
+          <t>10216012014</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>2014-10-10</t>
-        </is>
-      </c>
-      <c r="E41" s="7" t="inlineStr"/>
+          <t>2014-01-06</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
           <t>2014/15/16</t>
@@ -1661,20 +1797,24 @@
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>SNAYDER CAMPO</t>
+          <t>SEBASTIAN MATHIAS LUGO JIMENEZ</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>1012012001</t>
+          <t>1043479873</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr"/>
+          <t>2012-06-28</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
           <t>2012</t>
@@ -1692,23 +1832,27 @@
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>JAMED AMARANTO</t>
+          <t>DANY JOSE TAPIA SIERRA</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1137534185</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E43" s="7" t="inlineStr"/>
+          <t>2013-05-05</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>2014/15/16</t>
+          <t>2013</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
@@ -1723,12 +1867,12 @@
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>DEMIAN PEDROZA</t>
+          <t>GERONIMO RIVERA</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
@@ -1736,7 +1880,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="E44" s="5" t="inlineStr"/>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
           <t>2014/15/16</t>
@@ -1754,12 +1902,12 @@
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>STIVEN CABARCA</t>
+          <t>JESÚS DAVID AVILA ARIZA</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1194973338</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
@@ -1767,10 +1915,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="E45" s="7" t="inlineStr"/>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>2012</t>
+          <t>2014/15/16</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
@@ -1785,12 +1937,12 @@
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>YOJAINER VILLALOBOS</t>
+          <t>ENDERSON MARCANO</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>T001</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
@@ -1798,10 +1950,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="E46" s="5" t="inlineStr"/>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>2012</t>
+          <t>2014/15/16</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
@@ -1816,23 +1972,27 @@
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>ANDRES DAVID SOCARRAS CADENA</t>
+          <t>JAIR ANDRES MIRANDA CARO</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>1044655749</t>
+          <t>1047234329</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>2015-01-12</t>
-        </is>
-      </c>
-      <c r="E47" s="7" t="inlineStr"/>
+          <t>2012-12-13</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>2014/15/16</t>
+          <t>2012</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -1847,20 +2007,24 @@
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>ISRAEL BARRIOS</t>
+          <t>JAIR ANDRES MORENO ELLES</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1194976006</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr"/>
+          <t>2016-02-16</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
           <t>2014/15/16</t>
@@ -1878,12 +2042,12 @@
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>PEDROZA SNEYDER</t>
+          <t>TIAGO PRINS</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
@@ -1891,7 +2055,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="E49" s="7" t="inlineStr"/>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
           <t>2014/15/16</t>
@@ -1909,20 +2077,24 @@
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>GERONIMO RIVERA</t>
+          <t>CRISTIAN ALEXANDER MARCANO APARICIO</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>180914115</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr"/>
+          <t>2014-09-18</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
           <t>2014/15/16</t>
@@ -1940,23 +2112,27 @@
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>TIAGO PRINS</t>
+          <t>JOSEP DAVID ALDANA PUERTAS</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1043462171</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E51" s="7" t="inlineStr"/>
+          <t>2013-03-05</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>2014/15/16</t>
+          <t>2013</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
@@ -1971,23 +2147,27 @@
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>BRAYAN FERNANDEZ</t>
+          <t>YOJAINER JESUS VERA VILLALOBOS</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>300312673</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr"/>
+          <t>2012-03-03</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>2013</t>
+          <t>2012</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
@@ -2002,23 +2182,23 @@
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>DYLAN ALEJANDRO SÁNCHEZ CESPEDES</t>
+          <t>ISRAEL CAMAÑO</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>30528122012</t>
+          <t>1015016001</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>2012-12-28</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr"/>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>2012</t>
+          <t>2014/15/16</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
@@ -2033,17 +2213,17 @@
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>DANIEL LÓPEZ ROJO</t>
+          <t>MATEO DE JESUS BOSCAN GELVEZ</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>1046718667</t>
+          <t>1124517321</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>2013-10-04</t>
+          <t>2013-09-10</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr"/>
@@ -2064,23 +2244,23 @@
       </c>
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>JEIKHAM DAVID CAMAÑO OCHOA</t>
+          <t>MOISES EDUARDO CABALLERO CAÑAS</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>1194970988</t>
+          <t>1045251440</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>2013-07-23</t>
+          <t>2014-01-27</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr"/>
       <c r="F55" s="7" t="inlineStr">
         <is>
-          <t>2013</t>
+          <t>2014/15/16</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
@@ -2095,23 +2275,23 @@
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>RENE JUNIOR CERPA ALVAREZ</t>
+          <t>CARLOS ANDRES MORENO GARCIA</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>1044223163</t>
+          <t>1043696535</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>2013-08-15</t>
+          <t>2014-12-04</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr"/>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>2013</t>
+          <t>2014/15/16</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr">
@@ -2126,23 +2306,23 @@
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>CRISTIAN ALEXANDER MARCANO APARICIO</t>
+          <t>OSCAR DAVID LÓPEZ GARCIA</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>180914115</t>
+          <t>1043459628</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>2014-09-18</t>
+          <t>2012-08-03</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr"/>
       <c r="F57" s="7" t="inlineStr">
         <is>
-          <t>2014/15/16</t>
+          <t>2012</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
@@ -2157,23 +2337,23 @@
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>JOSE MIGUEL ALVAREZ CARRILLO</t>
+          <t>SANTIAGO HERNANDEZ GARCIA</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>1143252740</t>
+          <t>1043467436</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>2012-05-20</t>
+          <t>2014-10-10</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr"/>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>2012</t>
+          <t>2014/15/16</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr">
@@ -2188,17 +2368,17 @@
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>SANTIAGO ANDRES MENDOZA COLMENAREZ</t>
+          <t>SNAYDER CAMPO</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>9062012266</t>
+          <t>1012012001</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>2012-06-09</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr"/>
@@ -2219,17 +2399,17 @@
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>JHOAN ALEXANDER NAVARRO PLA</t>
+          <t>STIVEN CABARCA</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>1140869811</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>2012-06-22</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr"/>
@@ -2250,17 +2430,17 @@
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>LUIS EDUARDO CADENA SUAREZ</t>
+          <t>YOJAINER VILLALOBOS</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>1082352203</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>2012-04-23</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr"/>
@@ -2281,23 +2461,23 @@
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>ANTONY DAVID ARIZA ZAMORA</t>
+          <t>ISRAEL BARRIOS</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>04939456</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>2012-02-13</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr"/>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>2012</t>
+          <t>2014/15/16</t>
         </is>
       </c>
       <c r="G62" s="5" t="inlineStr">
@@ -2312,23 +2492,23 @@
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>JESUS ADRIAN TORRES RIOS</t>
+          <t>JEIKHAM DAVID CAMAÑO OCHOA</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>1041697767</t>
+          <t>1194970988</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>2012-01-20</t>
+          <t>2013-07-23</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr"/>
       <c r="F63" s="7" t="inlineStr">
         <is>
-          <t>2012</t>
+          <t>2013</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
@@ -2343,17 +2523,17 @@
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>JHONIER ARLES RONDON LUNA</t>
+          <t>JHOAN ALEXANDER NAVARRO PLA</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>1098763962</t>
+          <t>1140869811</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>2012-12-07</t>
+          <t>2012-06-22</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr"/>

</xml_diff>